<commit_message>
markers and markers base
</commit_message>
<xml_diff>
--- a/doc/notes.xlsx
+++ b/doc/notes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/renzosala/Develop/personal/tokeniko/doc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED19C436-4FC2-C549-9BC6-084192C8C6E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D129946-74A5-0C40-B9DB-E23C3E0E3F6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="22600" activeTab="6" xr2:uid="{ED098269-B10A-E440-BCE3-AF4955707036}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="22600" activeTab="7" xr2:uid="{ED098269-B10A-E440-BCE3-AF4955707036}"/>
   </bookViews>
   <sheets>
     <sheet name="General schema" sheetId="1" r:id="rId1"/>
@@ -20,6 +20,7 @@
     <sheet name="Test sheet Similarity" sheetId="4" r:id="rId5"/>
     <sheet name="Test sheet LL" sheetId="7" r:id="rId6"/>
     <sheet name="Compiler" sheetId="8" r:id="rId7"/>
+    <sheet name="Sheet1" sheetId="9" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="772" uniqueCount="458">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="778" uniqueCount="464">
   <si>
     <t>essere</t>
   </si>
@@ -1615,6 +1616,24 @@
   </si>
   <si>
     <t>isolate all the statements (across the nested structure) with duplication for conjuncts and subordinates, matching all entities</t>
+  </si>
+  <si>
+    <t>sentence</t>
+  </si>
+  <si>
+    <t>subject + properties</t>
+  </si>
+  <si>
+    <t>predicate + properties</t>
+  </si>
+  <si>
+    <t>direct + properties</t>
+  </si>
+  <si>
+    <t>ind (foreach type) + properties</t>
+  </si>
+  <si>
+    <t>100 + 2925</t>
   </si>
 </sst>
 </file>
@@ -2113,32 +2132,26 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2158,7 +2171,16 @@
     <xf numFmtId="0" fontId="15" fillId="3" borderId="9" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2173,29 +2195,26 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -2865,12 +2884,12 @@
       <c r="D30" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="E30" s="65" t="s">
+      <c r="E30" s="69" t="s">
         <v>127</v>
       </c>
-      <c r="F30" s="65"/>
-      <c r="G30" s="65"/>
-      <c r="H30" s="65"/>
+      <c r="F30" s="69"/>
+      <c r="G30" s="69"/>
+      <c r="H30" s="69"/>
       <c r="I30" s="4" t="s">
         <v>341</v>
       </c>
@@ -2933,12 +2952,12 @@
       <c r="D36" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="E36" s="65" t="s">
+      <c r="E36" s="69" t="s">
         <v>127</v>
       </c>
-      <c r="F36" s="65"/>
-      <c r="G36" s="65"/>
-      <c r="H36" s="65"/>
+      <c r="F36" s="69"/>
+      <c r="G36" s="69"/>
+      <c r="H36" s="69"/>
     </row>
     <row r="37" spans="2:10">
       <c r="B37" s="4"/>
@@ -3618,22 +3637,22 @@
       <c r="R5" s="19"/>
     </row>
     <row r="6" spans="3:21">
-      <c r="C6" s="68" t="s">
+      <c r="C6" s="76" t="s">
         <v>344</v>
       </c>
-      <c r="D6" s="69"/>
-      <c r="E6" s="69"/>
-      <c r="F6" s="69"/>
-      <c r="G6" s="69"/>
-      <c r="H6" s="69"/>
-      <c r="I6" s="69"/>
-      <c r="J6" s="69"/>
-      <c r="K6" s="69"/>
-      <c r="L6" s="69"/>
-      <c r="M6" s="69"/>
-      <c r="N6" s="69"/>
-      <c r="O6" s="69"/>
-      <c r="P6" s="70"/>
+      <c r="D6" s="77"/>
+      <c r="E6" s="77"/>
+      <c r="F6" s="77"/>
+      <c r="G6" s="77"/>
+      <c r="H6" s="77"/>
+      <c r="I6" s="77"/>
+      <c r="J6" s="77"/>
+      <c r="K6" s="77"/>
+      <c r="L6" s="77"/>
+      <c r="M6" s="77"/>
+      <c r="N6" s="77"/>
+      <c r="O6" s="77"/>
+      <c r="P6" s="78"/>
       <c r="Q6" s="22"/>
       <c r="R6" s="22" t="s">
         <v>218</v>
@@ -3641,24 +3660,24 @@
       <c r="U6" s="2"/>
     </row>
     <row r="7" spans="3:21">
-      <c r="C7" s="72" t="s">
+      <c r="C7" s="70" t="s">
         <v>227</v>
       </c>
-      <c r="D7" s="73"/>
-      <c r="E7" s="73"/>
-      <c r="F7" s="73"/>
-      <c r="G7" s="73"/>
-      <c r="H7" s="73"/>
-      <c r="I7" s="74"/>
-      <c r="J7" s="72" t="s">
+      <c r="D7" s="71"/>
+      <c r="E7" s="71"/>
+      <c r="F7" s="71"/>
+      <c r="G7" s="71"/>
+      <c r="H7" s="71"/>
+      <c r="I7" s="72"/>
+      <c r="J7" s="70" t="s">
         <v>230</v>
       </c>
-      <c r="K7" s="73"/>
-      <c r="L7" s="73"/>
-      <c r="M7" s="73"/>
-      <c r="N7" s="73"/>
-      <c r="O7" s="73"/>
-      <c r="P7" s="74"/>
+      <c r="K7" s="71"/>
+      <c r="L7" s="71"/>
+      <c r="M7" s="71"/>
+      <c r="N7" s="71"/>
+      <c r="O7" s="71"/>
+      <c r="P7" s="72"/>
       <c r="Q7" s="19"/>
       <c r="R7" s="19"/>
       <c r="U7" s="2"/>
@@ -3711,28 +3730,28 @@
       <c r="U8" s="2"/>
     </row>
     <row r="9" spans="3:21">
-      <c r="C9" s="79" t="s">
+      <c r="C9" s="80" t="s">
         <v>234</v>
       </c>
-      <c r="D9" s="68" t="b">
-        <v>1</v>
-      </c>
-      <c r="E9" s="69"/>
-      <c r="F9" s="69"/>
-      <c r="G9" s="69"/>
-      <c r="H9" s="69"/>
-      <c r="I9" s="70"/>
-      <c r="J9" s="79" t="s">
+      <c r="D9" s="76" t="b">
+        <v>1</v>
+      </c>
+      <c r="E9" s="77"/>
+      <c r="F9" s="77"/>
+      <c r="G9" s="77"/>
+      <c r="H9" s="77"/>
+      <c r="I9" s="78"/>
+      <c r="J9" s="80" t="s">
         <v>218</v>
       </c>
-      <c r="K9" s="67" t="b">
-        <v>1</v>
-      </c>
-      <c r="L9" s="67"/>
-      <c r="M9" s="67"/>
-      <c r="N9" s="67"/>
-      <c r="O9" s="67"/>
-      <c r="P9" s="67"/>
+      <c r="K9" s="79" t="b">
+        <v>1</v>
+      </c>
+      <c r="L9" s="79"/>
+      <c r="M9" s="79"/>
+      <c r="N9" s="79"/>
+      <c r="O9" s="79"/>
+      <c r="P9" s="79"/>
       <c r="Q9" s="24" t="b">
         <v>1</v>
       </c>
@@ -3748,24 +3767,24 @@
       </c>
     </row>
     <row r="10" spans="3:21">
-      <c r="C10" s="80"/>
-      <c r="D10" s="75" t="b">
-        <v>1</v>
-      </c>
-      <c r="E10" s="76"/>
-      <c r="F10" s="76"/>
-      <c r="G10" s="76"/>
-      <c r="H10" s="76"/>
-      <c r="I10" s="77"/>
-      <c r="J10" s="80"/>
-      <c r="K10" s="78" t="b">
-        <v>0</v>
-      </c>
-      <c r="L10" s="78"/>
-      <c r="M10" s="78"/>
-      <c r="N10" s="78"/>
-      <c r="O10" s="78"/>
-      <c r="P10" s="78"/>
+      <c r="C10" s="81"/>
+      <c r="D10" s="73" t="b">
+        <v>1</v>
+      </c>
+      <c r="E10" s="74"/>
+      <c r="F10" s="74"/>
+      <c r="G10" s="74"/>
+      <c r="H10" s="74"/>
+      <c r="I10" s="75"/>
+      <c r="J10" s="81"/>
+      <c r="K10" s="84" t="b">
+        <v>0</v>
+      </c>
+      <c r="L10" s="84"/>
+      <c r="M10" s="84"/>
+      <c r="N10" s="84"/>
+      <c r="O10" s="84"/>
+      <c r="P10" s="84"/>
       <c r="Q10" s="26" t="b">
         <v>0</v>
       </c>
@@ -3781,24 +3800,24 @@
       </c>
     </row>
     <row r="11" spans="3:21">
-      <c r="C11" s="80"/>
-      <c r="D11" s="68" t="b">
-        <v>0</v>
-      </c>
-      <c r="E11" s="69"/>
-      <c r="F11" s="69"/>
-      <c r="G11" s="69"/>
-      <c r="H11" s="69"/>
-      <c r="I11" s="70"/>
-      <c r="J11" s="80"/>
-      <c r="K11" s="67" t="b">
-        <v>1</v>
-      </c>
-      <c r="L11" s="67"/>
-      <c r="M11" s="67"/>
-      <c r="N11" s="67"/>
-      <c r="O11" s="67"/>
-      <c r="P11" s="67"/>
+      <c r="C11" s="81"/>
+      <c r="D11" s="76" t="b">
+        <v>0</v>
+      </c>
+      <c r="E11" s="77"/>
+      <c r="F11" s="77"/>
+      <c r="G11" s="77"/>
+      <c r="H11" s="77"/>
+      <c r="I11" s="78"/>
+      <c r="J11" s="81"/>
+      <c r="K11" s="79" t="b">
+        <v>1</v>
+      </c>
+      <c r="L11" s="79"/>
+      <c r="M11" s="79"/>
+      <c r="N11" s="79"/>
+      <c r="O11" s="79"/>
+      <c r="P11" s="79"/>
       <c r="Q11" s="24" t="b">
         <v>1</v>
       </c>
@@ -3814,24 +3833,24 @@
       </c>
     </row>
     <row r="12" spans="3:21">
-      <c r="C12" s="81"/>
-      <c r="D12" s="68" t="b">
-        <v>0</v>
-      </c>
-      <c r="E12" s="69"/>
-      <c r="F12" s="69"/>
-      <c r="G12" s="69"/>
-      <c r="H12" s="69"/>
-      <c r="I12" s="70"/>
-      <c r="J12" s="81"/>
-      <c r="K12" s="67" t="b">
-        <v>0</v>
-      </c>
-      <c r="L12" s="67"/>
-      <c r="M12" s="67"/>
-      <c r="N12" s="67"/>
-      <c r="O12" s="67"/>
-      <c r="P12" s="67"/>
+      <c r="C12" s="82"/>
+      <c r="D12" s="76" t="b">
+        <v>0</v>
+      </c>
+      <c r="E12" s="77"/>
+      <c r="F12" s="77"/>
+      <c r="G12" s="77"/>
+      <c r="H12" s="77"/>
+      <c r="I12" s="78"/>
+      <c r="J12" s="82"/>
+      <c r="K12" s="79" t="b">
+        <v>0</v>
+      </c>
+      <c r="L12" s="79"/>
+      <c r="M12" s="79"/>
+      <c r="N12" s="79"/>
+      <c r="O12" s="79"/>
+      <c r="P12" s="79"/>
       <c r="Q12" s="24" t="b">
         <v>1</v>
       </c>
@@ -3852,22 +3871,22 @@
       <c r="U13" s="2"/>
     </row>
     <row r="14" spans="3:21">
-      <c r="C14" s="68" t="s">
+      <c r="C14" s="76" t="s">
         <v>345</v>
       </c>
-      <c r="D14" s="69"/>
-      <c r="E14" s="69"/>
-      <c r="F14" s="69"/>
-      <c r="G14" s="69"/>
-      <c r="H14" s="69"/>
-      <c r="I14" s="69"/>
-      <c r="J14" s="69"/>
-      <c r="K14" s="69"/>
-      <c r="L14" s="69"/>
-      <c r="M14" s="69"/>
-      <c r="N14" s="69"/>
-      <c r="O14" s="69"/>
-      <c r="P14" s="70"/>
+      <c r="D14" s="77"/>
+      <c r="E14" s="77"/>
+      <c r="F14" s="77"/>
+      <c r="G14" s="77"/>
+      <c r="H14" s="77"/>
+      <c r="I14" s="77"/>
+      <c r="J14" s="77"/>
+      <c r="K14" s="77"/>
+      <c r="L14" s="77"/>
+      <c r="M14" s="77"/>
+      <c r="N14" s="77"/>
+      <c r="O14" s="77"/>
+      <c r="P14" s="78"/>
       <c r="Q14" s="19"/>
       <c r="R14" s="22" t="s">
         <v>219</v>
@@ -3875,24 +3894,24 @@
       <c r="U14" s="2"/>
     </row>
     <row r="15" spans="3:21">
-      <c r="C15" s="72" t="s">
+      <c r="C15" s="70" t="s">
         <v>228</v>
       </c>
-      <c r="D15" s="73"/>
-      <c r="E15" s="73"/>
-      <c r="F15" s="73"/>
-      <c r="G15" s="73"/>
-      <c r="H15" s="73"/>
-      <c r="I15" s="74"/>
-      <c r="J15" s="72" t="s">
+      <c r="D15" s="71"/>
+      <c r="E15" s="71"/>
+      <c r="F15" s="71"/>
+      <c r="G15" s="71"/>
+      <c r="H15" s="71"/>
+      <c r="I15" s="72"/>
+      <c r="J15" s="70" t="s">
         <v>230</v>
       </c>
-      <c r="K15" s="73"/>
-      <c r="L15" s="73"/>
-      <c r="M15" s="73"/>
-      <c r="N15" s="73"/>
-      <c r="O15" s="73"/>
-      <c r="P15" s="74"/>
+      <c r="K15" s="71"/>
+      <c r="L15" s="71"/>
+      <c r="M15" s="71"/>
+      <c r="N15" s="71"/>
+      <c r="O15" s="71"/>
+      <c r="P15" s="72"/>
       <c r="Q15" s="19"/>
       <c r="R15" s="19"/>
       <c r="U15" s="2"/>
@@ -3945,28 +3964,28 @@
       <c r="U16" s="2"/>
     </row>
     <row r="17" spans="3:21">
-      <c r="C17" s="79" t="s">
+      <c r="C17" s="80" t="s">
         <v>234</v>
       </c>
-      <c r="D17" s="68" t="b">
-        <v>1</v>
-      </c>
-      <c r="E17" s="69"/>
-      <c r="F17" s="69"/>
-      <c r="G17" s="69"/>
-      <c r="H17" s="69"/>
-      <c r="I17" s="70"/>
-      <c r="J17" s="79" t="s">
+      <c r="D17" s="76" t="b">
+        <v>1</v>
+      </c>
+      <c r="E17" s="77"/>
+      <c r="F17" s="77"/>
+      <c r="G17" s="77"/>
+      <c r="H17" s="77"/>
+      <c r="I17" s="78"/>
+      <c r="J17" s="80" t="s">
         <v>219</v>
       </c>
-      <c r="K17" s="67" t="b">
-        <v>1</v>
-      </c>
-      <c r="L17" s="67"/>
-      <c r="M17" s="67"/>
-      <c r="N17" s="67"/>
-      <c r="O17" s="67"/>
-      <c r="P17" s="67"/>
+      <c r="K17" s="79" t="b">
+        <v>1</v>
+      </c>
+      <c r="L17" s="79"/>
+      <c r="M17" s="79"/>
+      <c r="N17" s="79"/>
+      <c r="O17" s="79"/>
+      <c r="P17" s="79"/>
       <c r="Q17" s="24" t="b">
         <v>1</v>
       </c>
@@ -3974,24 +3993,24 @@
       <c r="U17" s="2"/>
     </row>
     <row r="18" spans="3:21">
-      <c r="C18" s="80"/>
-      <c r="D18" s="68" t="b">
-        <v>1</v>
-      </c>
-      <c r="E18" s="69"/>
-      <c r="F18" s="69"/>
-      <c r="G18" s="69"/>
-      <c r="H18" s="69"/>
-      <c r="I18" s="70"/>
-      <c r="J18" s="80"/>
-      <c r="K18" s="67" t="b">
-        <v>0</v>
-      </c>
-      <c r="L18" s="67"/>
-      <c r="M18" s="67"/>
-      <c r="N18" s="67"/>
-      <c r="O18" s="67"/>
-      <c r="P18" s="67"/>
+      <c r="C18" s="81"/>
+      <c r="D18" s="76" t="b">
+        <v>1</v>
+      </c>
+      <c r="E18" s="77"/>
+      <c r="F18" s="77"/>
+      <c r="G18" s="77"/>
+      <c r="H18" s="77"/>
+      <c r="I18" s="78"/>
+      <c r="J18" s="81"/>
+      <c r="K18" s="79" t="b">
+        <v>0</v>
+      </c>
+      <c r="L18" s="79"/>
+      <c r="M18" s="79"/>
+      <c r="N18" s="79"/>
+      <c r="O18" s="79"/>
+      <c r="P18" s="79"/>
       <c r="Q18" s="24" t="b">
         <v>1</v>
       </c>
@@ -3999,24 +4018,24 @@
       <c r="U18" s="2"/>
     </row>
     <row r="19" spans="3:21">
-      <c r="C19" s="80"/>
-      <c r="D19" s="75" t="b">
-        <v>0</v>
-      </c>
-      <c r="E19" s="76"/>
-      <c r="F19" s="76"/>
-      <c r="G19" s="76"/>
-      <c r="H19" s="76"/>
-      <c r="I19" s="77"/>
-      <c r="J19" s="80"/>
-      <c r="K19" s="78" t="b">
-        <v>1</v>
-      </c>
-      <c r="L19" s="78"/>
-      <c r="M19" s="78"/>
-      <c r="N19" s="78"/>
-      <c r="O19" s="78"/>
-      <c r="P19" s="78"/>
+      <c r="C19" s="81"/>
+      <c r="D19" s="73" t="b">
+        <v>0</v>
+      </c>
+      <c r="E19" s="74"/>
+      <c r="F19" s="74"/>
+      <c r="G19" s="74"/>
+      <c r="H19" s="74"/>
+      <c r="I19" s="75"/>
+      <c r="J19" s="81"/>
+      <c r="K19" s="84" t="b">
+        <v>1</v>
+      </c>
+      <c r="L19" s="84"/>
+      <c r="M19" s="84"/>
+      <c r="N19" s="84"/>
+      <c r="O19" s="84"/>
+      <c r="P19" s="84"/>
       <c r="Q19" s="26" t="b">
         <v>0</v>
       </c>
@@ -4024,24 +4043,24 @@
       <c r="U19" s="2"/>
     </row>
     <row r="20" spans="3:21">
-      <c r="C20" s="81"/>
-      <c r="D20" s="68" t="b">
-        <v>0</v>
-      </c>
-      <c r="E20" s="69"/>
-      <c r="F20" s="69"/>
-      <c r="G20" s="69"/>
-      <c r="H20" s="69"/>
-      <c r="I20" s="70"/>
-      <c r="J20" s="81"/>
-      <c r="K20" s="67" t="b">
-        <v>0</v>
-      </c>
-      <c r="L20" s="67"/>
-      <c r="M20" s="67"/>
-      <c r="N20" s="67"/>
-      <c r="O20" s="67"/>
-      <c r="P20" s="67"/>
+      <c r="C20" s="82"/>
+      <c r="D20" s="76" t="b">
+        <v>0</v>
+      </c>
+      <c r="E20" s="77"/>
+      <c r="F20" s="77"/>
+      <c r="G20" s="77"/>
+      <c r="H20" s="77"/>
+      <c r="I20" s="78"/>
+      <c r="J20" s="82"/>
+      <c r="K20" s="79" t="b">
+        <v>0</v>
+      </c>
+      <c r="L20" s="79"/>
+      <c r="M20" s="79"/>
+      <c r="N20" s="79"/>
+      <c r="O20" s="79"/>
+      <c r="P20" s="79"/>
       <c r="Q20" s="27" t="b">
         <v>1</v>
       </c>
@@ -4052,46 +4071,46 @@
       <c r="R21" s="19"/>
     </row>
     <row r="22" spans="3:21">
-      <c r="C22" s="68" t="s">
+      <c r="C22" s="76" t="s">
         <v>346</v>
       </c>
-      <c r="D22" s="69"/>
-      <c r="E22" s="69"/>
-      <c r="F22" s="69"/>
-      <c r="G22" s="69"/>
-      <c r="H22" s="69"/>
-      <c r="I22" s="69"/>
-      <c r="J22" s="69"/>
-      <c r="K22" s="69"/>
-      <c r="L22" s="69"/>
-      <c r="M22" s="69"/>
-      <c r="N22" s="69"/>
-      <c r="O22" s="69"/>
-      <c r="P22" s="70"/>
+      <c r="D22" s="77"/>
+      <c r="E22" s="77"/>
+      <c r="F22" s="77"/>
+      <c r="G22" s="77"/>
+      <c r="H22" s="77"/>
+      <c r="I22" s="77"/>
+      <c r="J22" s="77"/>
+      <c r="K22" s="77"/>
+      <c r="L22" s="77"/>
+      <c r="M22" s="77"/>
+      <c r="N22" s="77"/>
+      <c r="O22" s="77"/>
+      <c r="P22" s="78"/>
       <c r="Q22" s="19"/>
       <c r="R22" s="22" t="s">
         <v>217</v>
       </c>
     </row>
     <row r="23" spans="3:21">
-      <c r="C23" s="72" t="s">
+      <c r="C23" s="70" t="s">
         <v>229</v>
       </c>
-      <c r="D23" s="73"/>
-      <c r="E23" s="73"/>
-      <c r="F23" s="73"/>
-      <c r="G23" s="73"/>
-      <c r="H23" s="73"/>
-      <c r="I23" s="74"/>
-      <c r="J23" s="72" t="s">
+      <c r="D23" s="71"/>
+      <c r="E23" s="71"/>
+      <c r="F23" s="71"/>
+      <c r="G23" s="71"/>
+      <c r="H23" s="71"/>
+      <c r="I23" s="72"/>
+      <c r="J23" s="70" t="s">
         <v>231</v>
       </c>
-      <c r="K23" s="73"/>
-      <c r="L23" s="73"/>
-      <c r="M23" s="73"/>
-      <c r="N23" s="73"/>
-      <c r="O23" s="73"/>
-      <c r="P23" s="74"/>
+      <c r="K23" s="71"/>
+      <c r="L23" s="71"/>
+      <c r="M23" s="71"/>
+      <c r="N23" s="71"/>
+      <c r="O23" s="71"/>
+      <c r="P23" s="72"/>
       <c r="Q23" s="19"/>
       <c r="R23" s="19"/>
     </row>
@@ -4142,100 +4161,100 @@
       <c r="R24" s="19"/>
     </row>
     <row r="25" spans="3:21">
-      <c r="C25" s="79" t="s">
+      <c r="C25" s="80" t="s">
         <v>234</v>
       </c>
-      <c r="D25" s="68" t="b">
-        <v>1</v>
-      </c>
-      <c r="E25" s="69"/>
-      <c r="F25" s="69"/>
-      <c r="G25" s="69"/>
-      <c r="H25" s="69"/>
-      <c r="I25" s="70"/>
-      <c r="J25" s="82" t="s">
+      <c r="D25" s="76" t="b">
+        <v>1</v>
+      </c>
+      <c r="E25" s="77"/>
+      <c r="F25" s="77"/>
+      <c r="G25" s="77"/>
+      <c r="H25" s="77"/>
+      <c r="I25" s="78"/>
+      <c r="J25" s="83" t="s">
         <v>233</v>
       </c>
-      <c r="K25" s="67" t="b">
-        <v>1</v>
-      </c>
-      <c r="L25" s="67"/>
-      <c r="M25" s="67"/>
-      <c r="N25" s="67"/>
-      <c r="O25" s="67"/>
-      <c r="P25" s="67"/>
+      <c r="K25" s="79" t="b">
+        <v>1</v>
+      </c>
+      <c r="L25" s="79"/>
+      <c r="M25" s="79"/>
+      <c r="N25" s="79"/>
+      <c r="O25" s="79"/>
+      <c r="P25" s="79"/>
       <c r="Q25" s="24" t="b">
         <v>1</v>
       </c>
       <c r="R25" s="19"/>
     </row>
     <row r="26" spans="3:21">
-      <c r="C26" s="80"/>
-      <c r="D26" s="75" t="b">
-        <v>1</v>
-      </c>
-      <c r="E26" s="76"/>
-      <c r="F26" s="76"/>
-      <c r="G26" s="76"/>
-      <c r="H26" s="76"/>
-      <c r="I26" s="77"/>
-      <c r="J26" s="80"/>
-      <c r="K26" s="78" t="b">
-        <v>0</v>
-      </c>
-      <c r="L26" s="78"/>
-      <c r="M26" s="78"/>
-      <c r="N26" s="78"/>
-      <c r="O26" s="78"/>
-      <c r="P26" s="78"/>
+      <c r="C26" s="81"/>
+      <c r="D26" s="73" t="b">
+        <v>1</v>
+      </c>
+      <c r="E26" s="74"/>
+      <c r="F26" s="74"/>
+      <c r="G26" s="74"/>
+      <c r="H26" s="74"/>
+      <c r="I26" s="75"/>
+      <c r="J26" s="81"/>
+      <c r="K26" s="84" t="b">
+        <v>0</v>
+      </c>
+      <c r="L26" s="84"/>
+      <c r="M26" s="84"/>
+      <c r="N26" s="84"/>
+      <c r="O26" s="84"/>
+      <c r="P26" s="84"/>
       <c r="Q26" s="26" t="b">
         <v>0</v>
       </c>
       <c r="R26" s="19"/>
     </row>
     <row r="27" spans="3:21">
-      <c r="C27" s="80"/>
-      <c r="D27" s="75" t="b">
-        <v>0</v>
-      </c>
-      <c r="E27" s="76"/>
-      <c r="F27" s="76"/>
-      <c r="G27" s="76"/>
-      <c r="H27" s="76"/>
-      <c r="I27" s="77"/>
-      <c r="J27" s="80"/>
-      <c r="K27" s="78" t="b">
-        <v>1</v>
-      </c>
-      <c r="L27" s="78"/>
-      <c r="M27" s="78"/>
-      <c r="N27" s="78"/>
-      <c r="O27" s="78"/>
-      <c r="P27" s="78"/>
+      <c r="C27" s="81"/>
+      <c r="D27" s="73" t="b">
+        <v>0</v>
+      </c>
+      <c r="E27" s="74"/>
+      <c r="F27" s="74"/>
+      <c r="G27" s="74"/>
+      <c r="H27" s="74"/>
+      <c r="I27" s="75"/>
+      <c r="J27" s="81"/>
+      <c r="K27" s="84" t="b">
+        <v>1</v>
+      </c>
+      <c r="L27" s="84"/>
+      <c r="M27" s="84"/>
+      <c r="N27" s="84"/>
+      <c r="O27" s="84"/>
+      <c r="P27" s="84"/>
       <c r="Q27" s="28" t="b">
         <v>0</v>
       </c>
       <c r="R27" s="19"/>
     </row>
     <row r="28" spans="3:21">
-      <c r="C28" s="81"/>
-      <c r="D28" s="68" t="b">
-        <v>0</v>
-      </c>
-      <c r="E28" s="69"/>
-      <c r="F28" s="69"/>
-      <c r="G28" s="69"/>
-      <c r="H28" s="69"/>
-      <c r="I28" s="70"/>
-      <c r="J28" s="81"/>
-      <c r="K28" s="67" t="b">
-        <v>0</v>
-      </c>
-      <c r="L28" s="67"/>
-      <c r="M28" s="67"/>
-      <c r="N28" s="67"/>
-      <c r="O28" s="67"/>
-      <c r="P28" s="67"/>
+      <c r="C28" s="82"/>
+      <c r="D28" s="76" t="b">
+        <v>0</v>
+      </c>
+      <c r="E28" s="77"/>
+      <c r="F28" s="77"/>
+      <c r="G28" s="77"/>
+      <c r="H28" s="77"/>
+      <c r="I28" s="78"/>
+      <c r="J28" s="82"/>
+      <c r="K28" s="79" t="b">
+        <v>0</v>
+      </c>
+      <c r="L28" s="79"/>
+      <c r="M28" s="79"/>
+      <c r="N28" s="79"/>
+      <c r="O28" s="79"/>
+      <c r="P28" s="79"/>
       <c r="Q28" s="27" t="b">
         <v>1</v>
       </c>
@@ -4245,46 +4264,46 @@
       <c r="R29" s="19"/>
     </row>
     <row r="30" spans="3:21">
-      <c r="C30" s="68" t="s">
+      <c r="C30" s="76" t="s">
         <v>347</v>
       </c>
-      <c r="D30" s="69"/>
-      <c r="E30" s="69"/>
-      <c r="F30" s="69"/>
-      <c r="G30" s="69"/>
-      <c r="H30" s="69"/>
-      <c r="I30" s="69"/>
-      <c r="J30" s="69"/>
-      <c r="K30" s="69"/>
-      <c r="L30" s="69"/>
-      <c r="M30" s="69"/>
-      <c r="N30" s="69"/>
-      <c r="O30" s="69"/>
-      <c r="P30" s="70"/>
+      <c r="D30" s="77"/>
+      <c r="E30" s="77"/>
+      <c r="F30" s="77"/>
+      <c r="G30" s="77"/>
+      <c r="H30" s="77"/>
+      <c r="I30" s="77"/>
+      <c r="J30" s="77"/>
+      <c r="K30" s="77"/>
+      <c r="L30" s="77"/>
+      <c r="M30" s="77"/>
+      <c r="N30" s="77"/>
+      <c r="O30" s="77"/>
+      <c r="P30" s="78"/>
       <c r="Q30" s="19"/>
       <c r="R30" s="22" t="s">
         <v>220</v>
       </c>
     </row>
     <row r="31" spans="3:21">
-      <c r="C31" s="72" t="s">
+      <c r="C31" s="70" t="s">
         <v>237</v>
       </c>
-      <c r="D31" s="73"/>
-      <c r="E31" s="73"/>
-      <c r="F31" s="73"/>
-      <c r="G31" s="73"/>
-      <c r="H31" s="73"/>
-      <c r="I31" s="74"/>
-      <c r="J31" s="72" t="s">
+      <c r="D31" s="71"/>
+      <c r="E31" s="71"/>
+      <c r="F31" s="71"/>
+      <c r="G31" s="71"/>
+      <c r="H31" s="71"/>
+      <c r="I31" s="72"/>
+      <c r="J31" s="70" t="s">
         <v>238</v>
       </c>
-      <c r="K31" s="73"/>
-      <c r="L31" s="73"/>
-      <c r="M31" s="73"/>
-      <c r="N31" s="73"/>
-      <c r="O31" s="73"/>
-      <c r="P31" s="74"/>
+      <c r="K31" s="71"/>
+      <c r="L31" s="71"/>
+      <c r="M31" s="71"/>
+      <c r="N31" s="71"/>
+      <c r="O31" s="71"/>
+      <c r="P31" s="72"/>
       <c r="Q31" s="19"/>
       <c r="R31" s="19"/>
     </row>
@@ -4338,25 +4357,25 @@
       <c r="C33" s="24" t="s">
         <v>236</v>
       </c>
-      <c r="D33" s="68" t="s">
+      <c r="D33" s="76" t="s">
         <v>216</v>
       </c>
-      <c r="E33" s="69"/>
-      <c r="F33" s="69"/>
-      <c r="G33" s="69"/>
-      <c r="H33" s="69"/>
-      <c r="I33" s="70"/>
+      <c r="E33" s="77"/>
+      <c r="F33" s="77"/>
+      <c r="G33" s="77"/>
+      <c r="H33" s="77"/>
+      <c r="I33" s="78"/>
       <c r="J33" s="24" t="s">
         <v>235</v>
       </c>
-      <c r="K33" s="67" t="s">
+      <c r="K33" s="79" t="s">
         <v>221</v>
       </c>
-      <c r="L33" s="67"/>
-      <c r="M33" s="67"/>
-      <c r="N33" s="67"/>
-      <c r="O33" s="67"/>
-      <c r="P33" s="67"/>
+      <c r="L33" s="79"/>
+      <c r="M33" s="79"/>
+      <c r="N33" s="79"/>
+      <c r="O33" s="79"/>
+      <c r="P33" s="79"/>
       <c r="Q33" s="24" t="s">
         <v>239</v>
       </c>
@@ -4370,19 +4389,19 @@
     <row r="36" spans="3:21" ht="26">
       <c r="C36" s="20"/>
       <c r="D36" s="20"/>
-      <c r="F36" s="71" t="s">
+      <c r="F36" s="86" t="s">
         <v>253</v>
       </c>
-      <c r="G36" s="71"/>
-      <c r="H36" s="71"/>
-      <c r="I36" s="71"/>
-      <c r="J36" s="71"/>
-      <c r="K36" s="71"/>
-      <c r="L36" s="71"/>
-      <c r="M36" s="71"/>
-      <c r="N36" s="71"/>
-      <c r="O36" s="71"/>
-      <c r="P36" s="71"/>
+      <c r="G36" s="86"/>
+      <c r="H36" s="86"/>
+      <c r="I36" s="86"/>
+      <c r="J36" s="86"/>
+      <c r="K36" s="86"/>
+      <c r="L36" s="86"/>
+      <c r="M36" s="86"/>
+      <c r="N36" s="86"/>
+      <c r="O36" s="86"/>
+      <c r="P36" s="86"/>
     </row>
     <row r="37" spans="3:21">
       <c r="C37" s="30" t="s">
@@ -4664,18 +4683,18 @@
       </c>
     </row>
     <row r="64" spans="2:12">
-      <c r="C64" s="66" t="s">
+      <c r="C64" s="85" t="s">
         <v>286</v>
       </c>
-      <c r="D64" s="66"/>
-      <c r="E64" s="66"/>
-      <c r="F64" s="66"/>
-      <c r="G64" s="66"/>
-      <c r="H64" s="66"/>
-      <c r="I64" s="66"/>
-      <c r="J64" s="66"/>
-      <c r="K64" s="66"/>
-      <c r="L64" s="66"/>
+      <c r="D64" s="85"/>
+      <c r="E64" s="85"/>
+      <c r="F64" s="85"/>
+      <c r="G64" s="85"/>
+      <c r="H64" s="85"/>
+      <c r="I64" s="85"/>
+      <c r="J64" s="85"/>
+      <c r="K64" s="85"/>
+      <c r="L64" s="85"/>
     </row>
     <row r="65" spans="3:12">
       <c r="C65" s="19" t="b">
@@ -4833,18 +4852,18 @@
       <c r="G69" s="19"/>
     </row>
     <row r="70" spans="3:12">
-      <c r="C70" s="66" t="s">
+      <c r="C70" s="85" t="s">
         <v>287</v>
       </c>
-      <c r="D70" s="66"/>
-      <c r="E70" s="66"/>
-      <c r="F70" s="66"/>
-      <c r="G70" s="66"/>
-      <c r="H70" s="66"/>
-      <c r="I70" s="66"/>
-      <c r="J70" s="66"/>
-      <c r="K70" s="66"/>
-      <c r="L70" s="66"/>
+      <c r="D70" s="85"/>
+      <c r="E70" s="85"/>
+      <c r="F70" s="85"/>
+      <c r="G70" s="85"/>
+      <c r="H70" s="85"/>
+      <c r="I70" s="85"/>
+      <c r="J70" s="85"/>
+      <c r="K70" s="85"/>
+      <c r="L70" s="85"/>
     </row>
     <row r="71" spans="3:12">
       <c r="C71" s="19">
@@ -5167,18 +5186,18 @@
       </c>
     </row>
     <row r="80" spans="3:12">
-      <c r="C80" s="66" t="s">
+      <c r="C80" s="85" t="s">
         <v>299</v>
       </c>
-      <c r="D80" s="66"/>
-      <c r="E80" s="66"/>
-      <c r="F80" s="66"/>
-      <c r="G80" s="66"/>
-      <c r="H80" s="66"/>
-      <c r="I80" s="66"/>
-      <c r="J80" s="66"/>
-      <c r="K80" s="66"/>
-      <c r="L80" s="66"/>
+      <c r="D80" s="85"/>
+      <c r="E80" s="85"/>
+      <c r="F80" s="85"/>
+      <c r="G80" s="85"/>
+      <c r="H80" s="85"/>
+      <c r="I80" s="85"/>
+      <c r="J80" s="85"/>
+      <c r="K80" s="85"/>
+      <c r="L80" s="85"/>
     </row>
     <row r="81" spans="3:14">
       <c r="C81" s="19">
@@ -5692,6 +5711,38 @@
     </row>
   </sheetData>
   <mergeCells count="48">
+    <mergeCell ref="C80:L80"/>
+    <mergeCell ref="C64:L64"/>
+    <mergeCell ref="C70:L70"/>
+    <mergeCell ref="K33:P33"/>
+    <mergeCell ref="D33:I33"/>
+    <mergeCell ref="F36:P36"/>
+    <mergeCell ref="C7:I7"/>
+    <mergeCell ref="D12:I12"/>
+    <mergeCell ref="D11:I11"/>
+    <mergeCell ref="D10:I10"/>
+    <mergeCell ref="D9:I9"/>
+    <mergeCell ref="C22:P22"/>
+    <mergeCell ref="K9:P9"/>
+    <mergeCell ref="K10:P10"/>
+    <mergeCell ref="K11:P11"/>
+    <mergeCell ref="K12:P12"/>
+    <mergeCell ref="C6:P6"/>
+    <mergeCell ref="J9:J12"/>
+    <mergeCell ref="J25:J28"/>
+    <mergeCell ref="J17:J20"/>
+    <mergeCell ref="D25:I25"/>
+    <mergeCell ref="C9:C12"/>
+    <mergeCell ref="C17:C20"/>
+    <mergeCell ref="C25:C28"/>
+    <mergeCell ref="K25:P25"/>
+    <mergeCell ref="K26:P26"/>
+    <mergeCell ref="K27:P27"/>
+    <mergeCell ref="K28:P28"/>
+    <mergeCell ref="C14:P14"/>
+    <mergeCell ref="K17:P17"/>
+    <mergeCell ref="K18:P18"/>
+    <mergeCell ref="K19:P19"/>
     <mergeCell ref="J31:P31"/>
     <mergeCell ref="J23:P23"/>
     <mergeCell ref="J7:P7"/>
@@ -5708,38 +5759,6 @@
     <mergeCell ref="C23:I23"/>
     <mergeCell ref="C31:I31"/>
     <mergeCell ref="C30:P30"/>
-    <mergeCell ref="C6:P6"/>
-    <mergeCell ref="J9:J12"/>
-    <mergeCell ref="J25:J28"/>
-    <mergeCell ref="J17:J20"/>
-    <mergeCell ref="D25:I25"/>
-    <mergeCell ref="C9:C12"/>
-    <mergeCell ref="C17:C20"/>
-    <mergeCell ref="C25:C28"/>
-    <mergeCell ref="K25:P25"/>
-    <mergeCell ref="K26:P26"/>
-    <mergeCell ref="K27:P27"/>
-    <mergeCell ref="K28:P28"/>
-    <mergeCell ref="C14:P14"/>
-    <mergeCell ref="K17:P17"/>
-    <mergeCell ref="K18:P18"/>
-    <mergeCell ref="K19:P19"/>
-    <mergeCell ref="C22:P22"/>
-    <mergeCell ref="K9:P9"/>
-    <mergeCell ref="K10:P10"/>
-    <mergeCell ref="K11:P11"/>
-    <mergeCell ref="K12:P12"/>
-    <mergeCell ref="C7:I7"/>
-    <mergeCell ref="D12:I12"/>
-    <mergeCell ref="D11:I11"/>
-    <mergeCell ref="D10:I10"/>
-    <mergeCell ref="D9:I9"/>
-    <mergeCell ref="C80:L80"/>
-    <mergeCell ref="C64:L64"/>
-    <mergeCell ref="C70:L70"/>
-    <mergeCell ref="K33:P33"/>
-    <mergeCell ref="D33:I33"/>
-    <mergeCell ref="F36:P36"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -5833,62 +5852,62 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:33">
-      <c r="B2" s="83" t="s">
+      <c r="B2" s="87" t="s">
         <v>68</v>
       </c>
-      <c r="C2" s="83"/>
-      <c r="D2" s="83"/>
-      <c r="E2" s="83"/>
+      <c r="C2" s="87"/>
+      <c r="D2" s="87"/>
+      <c r="E2" s="87"/>
     </row>
     <row r="3" spans="2:33">
-      <c r="B3" s="83"/>
-      <c r="C3" s="83"/>
-      <c r="D3" s="83"/>
-      <c r="E3" s="83"/>
+      <c r="B3" s="87"/>
+      <c r="C3" s="87"/>
+      <c r="D3" s="87"/>
+      <c r="E3" s="87"/>
       <c r="M3" s="31"/>
     </row>
     <row r="4" spans="2:33">
-      <c r="B4" s="83"/>
-      <c r="C4" s="83"/>
-      <c r="D4" s="83"/>
-      <c r="E4" s="83"/>
+      <c r="B4" s="87"/>
+      <c r="C4" s="87"/>
+      <c r="D4" s="87"/>
+      <c r="E4" s="87"/>
     </row>
     <row r="5" spans="2:33">
-      <c r="B5" s="83"/>
-      <c r="C5" s="83"/>
-      <c r="D5" s="83"/>
-      <c r="E5" s="83"/>
+      <c r="B5" s="87"/>
+      <c r="C5" s="87"/>
+      <c r="D5" s="87"/>
+      <c r="E5" s="87"/>
     </row>
     <row r="6" spans="2:33">
-      <c r="B6" s="83"/>
-      <c r="C6" s="83"/>
-      <c r="D6" s="83"/>
-      <c r="E6" s="83"/>
-      <c r="O6" s="83" t="s">
+      <c r="B6" s="87"/>
+      <c r="C6" s="87"/>
+      <c r="D6" s="87"/>
+      <c r="E6" s="87"/>
+      <c r="O6" s="87" t="s">
         <v>33</v>
       </c>
-      <c r="P6" s="83"/>
-      <c r="Q6" s="83"/>
-      <c r="R6" s="83"/>
+      <c r="P6" s="87"/>
+      <c r="Q6" s="87"/>
+      <c r="R6" s="87"/>
     </row>
     <row r="7" spans="2:33">
-      <c r="O7" s="83"/>
-      <c r="P7" s="83"/>
-      <c r="Q7" s="83"/>
-      <c r="R7" s="83"/>
+      <c r="O7" s="87"/>
+      <c r="P7" s="87"/>
+      <c r="Q7" s="87"/>
+      <c r="R7" s="87"/>
     </row>
     <row r="8" spans="2:33">
-      <c r="C8" s="84" t="s">
+      <c r="C8" s="88" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="84"/>
-      <c r="E8" s="84"/>
-      <c r="F8" s="84"/>
-      <c r="G8" s="84"/>
-      <c r="O8" s="83"/>
-      <c r="P8" s="83"/>
-      <c r="Q8" s="83"/>
-      <c r="R8" s="83"/>
+      <c r="D8" s="88"/>
+      <c r="E8" s="88"/>
+      <c r="F8" s="88"/>
+      <c r="G8" s="88"/>
+      <c r="O8" s="87"/>
+      <c r="P8" s="87"/>
+      <c r="Q8" s="87"/>
+      <c r="R8" s="87"/>
     </row>
     <row r="9" spans="2:33">
       <c r="B9" s="33" t="s">
@@ -5919,10 +5938,10 @@
         <v>6</v>
       </c>
       <c r="L9" s="31"/>
-      <c r="O9" s="83"/>
-      <c r="P9" s="83"/>
-      <c r="Q9" s="83"/>
-      <c r="R9" s="83"/>
+      <c r="O9" s="87"/>
+      <c r="P9" s="87"/>
+      <c r="Q9" s="87"/>
+      <c r="R9" s="87"/>
     </row>
     <row r="10" spans="2:33">
       <c r="B10" s="31" t="s">
@@ -5952,10 +5971,10 @@
       <c r="J10" s="2">
         <v>0</v>
       </c>
-      <c r="O10" s="83"/>
-      <c r="P10" s="83"/>
-      <c r="Q10" s="83"/>
-      <c r="R10" s="83"/>
+      <c r="O10" s="87"/>
+      <c r="P10" s="87"/>
+      <c r="Q10" s="87"/>
+      <c r="R10" s="87"/>
     </row>
     <row r="11" spans="2:33">
       <c r="B11" s="31" t="s">
@@ -6824,12 +6843,12 @@
       </c>
     </row>
     <row r="25" spans="2:33">
-      <c r="B25" s="83" t="s">
+      <c r="B25" s="87" t="s">
         <v>69</v>
       </c>
-      <c r="C25" s="83"/>
-      <c r="D25" s="83"/>
-      <c r="E25" s="83"/>
+      <c r="C25" s="87"/>
+      <c r="D25" s="87"/>
+      <c r="E25" s="87"/>
       <c r="O25" s="2" t="s">
         <v>23</v>
       </c>
@@ -6898,10 +6917,10 @@
       </c>
     </row>
     <row r="26" spans="2:33" ht="16" customHeight="1">
-      <c r="B26" s="83"/>
-      <c r="C26" s="83"/>
-      <c r="D26" s="83"/>
-      <c r="E26" s="83"/>
+      <c r="B26" s="87"/>
+      <c r="C26" s="87"/>
+      <c r="D26" s="87"/>
+      <c r="E26" s="87"/>
       <c r="N26" s="34" t="s">
         <v>23</v>
       </c>
@@ -6972,10 +6991,10 @@
       </c>
     </row>
     <row r="27" spans="2:33" ht="16" customHeight="1">
-      <c r="B27" s="83"/>
-      <c r="C27" s="83"/>
-      <c r="D27" s="83"/>
-      <c r="E27" s="83"/>
+      <c r="B27" s="87"/>
+      <c r="C27" s="87"/>
+      <c r="D27" s="87"/>
+      <c r="E27" s="87"/>
       <c r="N27" s="34" t="s">
         <v>24</v>
       </c>
@@ -7046,10 +7065,10 @@
       </c>
     </row>
     <row r="28" spans="2:33" ht="16" customHeight="1">
-      <c r="B28" s="83"/>
-      <c r="C28" s="83"/>
-      <c r="D28" s="83"/>
-      <c r="E28" s="83"/>
+      <c r="B28" s="87"/>
+      <c r="C28" s="87"/>
+      <c r="D28" s="87"/>
+      <c r="E28" s="87"/>
       <c r="N28" s="34" t="s">
         <v>25</v>
       </c>
@@ -7120,10 +7139,10 @@
       </c>
     </row>
     <row r="29" spans="2:33" ht="16" customHeight="1">
-      <c r="B29" s="83"/>
-      <c r="C29" s="83"/>
-      <c r="D29" s="83"/>
-      <c r="E29" s="83"/>
+      <c r="B29" s="87"/>
+      <c r="C29" s="87"/>
+      <c r="D29" s="87"/>
+      <c r="E29" s="87"/>
       <c r="N29" s="34" t="s">
         <v>27</v>
       </c>
@@ -8607,7 +8626,7 @@
       <c r="M18" s="6"/>
     </row>
     <row r="19" spans="1:15" ht="39" customHeight="1">
-      <c r="A19" s="63">
+      <c r="A19" s="89">
         <v>2</v>
       </c>
       <c r="B19" s="6" t="s">
@@ -8651,7 +8670,7 @@
       </c>
     </row>
     <row r="20" spans="1:15" ht="39" customHeight="1">
-      <c r="A20" s="63"/>
+      <c r="A20" s="89"/>
       <c r="B20" s="6" t="s">
         <v>98</v>
       </c>
@@ -8870,12 +8889,12 @@
       <c r="F29" s="6"/>
       <c r="G29" s="6"/>
       <c r="H29" s="6"/>
-      <c r="I29" s="64" t="s">
+      <c r="I29" s="90" t="s">
         <v>419</v>
       </c>
-      <c r="J29" s="64"/>
-      <c r="K29" s="64"/>
-      <c r="L29" s="64"/>
+      <c r="J29" s="90"/>
+      <c r="K29" s="90"/>
+      <c r="L29" s="90"/>
     </row>
     <row r="30" spans="1:15" ht="39" customHeight="1">
       <c r="A30" s="6"/>
@@ -9240,12 +9259,12 @@
       <c r="F47" s="6"/>
       <c r="G47" s="6"/>
       <c r="H47" s="6"/>
-      <c r="I47" s="64" t="s">
+      <c r="I47" s="90" t="s">
         <v>420</v>
       </c>
-      <c r="J47" s="64"/>
-      <c r="K47" s="64"/>
-      <c r="L47" s="64"/>
+      <c r="J47" s="90"/>
+      <c r="K47" s="90"/>
+      <c r="L47" s="90"/>
       <c r="M47" s="6"/>
       <c r="N47" s="6"/>
     </row>
@@ -9525,17 +9544,17 @@
   <dimension ref="B2:J21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col min="2" max="2" width="4.5" style="85" customWidth="1"/>
-    <col min="9" max="9" width="4.33203125" style="89" customWidth="1"/>
+    <col min="2" max="2" width="4.5" style="63" customWidth="1"/>
+    <col min="9" max="9" width="4.33203125" style="67" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:10" ht="26">
-      <c r="B2" s="87" t="s">
+      <c r="B2" s="65" t="s">
         <v>440</v>
       </c>
     </row>
     <row r="4" spans="2:10">
-      <c r="B4" s="88" t="s">
+      <c r="B4" s="66" t="s">
         <v>441</v>
       </c>
     </row>
@@ -9543,18 +9562,18 @@
       <c r="C5" t="s">
         <v>444</v>
       </c>
-      <c r="I5" s="90" t="s">
+      <c r="I5" s="68" t="s">
         <v>450</v>
       </c>
     </row>
     <row r="7" spans="2:10">
-      <c r="B7" s="85">
+      <c r="B7" s="63">
         <v>1</v>
       </c>
       <c r="C7" t="s">
         <v>443</v>
       </c>
-      <c r="I7" s="89">
+      <c r="I7" s="67">
         <v>1</v>
       </c>
       <c r="J7" t="s">
@@ -9562,13 +9581,13 @@
       </c>
     </row>
     <row r="8" spans="2:10">
-      <c r="B8" s="85">
+      <c r="B8" s="63">
         <v>2</v>
       </c>
       <c r="C8" t="s">
         <v>453</v>
       </c>
-      <c r="I8" s="89">
+      <c r="I8" s="67">
         <v>2</v>
       </c>
       <c r="J8" t="s">
@@ -9576,7 +9595,7 @@
       </c>
     </row>
     <row r="9" spans="2:10">
-      <c r="B9" s="85">
+      <c r="B9" s="63">
         <v>3</v>
       </c>
       <c r="C9" t="s">
@@ -9584,7 +9603,7 @@
       </c>
     </row>
     <row r="10" spans="2:10">
-      <c r="B10" s="85">
+      <c r="B10" s="63">
         <v>4</v>
       </c>
       <c r="C10" t="s">
@@ -9597,7 +9616,7 @@
       </c>
     </row>
     <row r="14" spans="2:10">
-      <c r="B14" s="85">
+      <c r="B14" s="63">
         <v>1</v>
       </c>
       <c r="C14" t="s">
@@ -9605,7 +9624,7 @@
       </c>
     </row>
     <row r="15" spans="2:10">
-      <c r="B15" s="85">
+      <c r="B15" s="63">
         <v>2</v>
       </c>
       <c r="C15" t="s">
@@ -9613,7 +9632,7 @@
       </c>
     </row>
     <row r="16" spans="2:10">
-      <c r="B16" s="85">
+      <c r="B16" s="63">
         <v>3</v>
       </c>
       <c r="C16" t="s">
@@ -9621,12 +9640,12 @@
       </c>
     </row>
     <row r="18" spans="2:3">
-      <c r="B18" s="86" t="s">
+      <c r="B18" s="64" t="s">
         <v>449</v>
       </c>
     </row>
     <row r="19" spans="2:3">
-      <c r="B19" s="85">
+      <c r="B19" s="63">
         <v>1</v>
       </c>
       <c r="C19" t="s">
@@ -9634,7 +9653,7 @@
       </c>
     </row>
     <row r="20" spans="2:3">
-      <c r="B20" s="85">
+      <c r="B20" s="63">
         <v>2</v>
       </c>
       <c r="C20" t="s">
@@ -9642,11 +9661,59 @@
       </c>
     </row>
     <row r="21" spans="2:3">
-      <c r="B21" s="85">
+      <c r="B21" s="63">
         <v>3</v>
       </c>
       <c r="C21" t="s">
         <v>456</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8DD2502-0F1B-8E4C-91C2-32C74D9C1A25}">
+  <dimension ref="B4:E8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <cols>
+    <col min="2" max="2" width="20.1640625" customWidth="1"/>
+    <col min="3" max="3" width="20.33203125" customWidth="1"/>
+    <col min="4" max="4" width="19.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="2:5">
+      <c r="B4" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="6" spans="2:5">
+      <c r="B6" t="s">
+        <v>459</v>
+      </c>
+      <c r="C6" t="s">
+        <v>460</v>
+      </c>
+      <c r="D6" t="s">
+        <v>461</v>
+      </c>
+      <c r="E6" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5">
+      <c r="B8">
+        <v>2925</v>
+      </c>
+      <c r="C8">
+        <v>2925</v>
+      </c>
+      <c r="D8">
+        <v>2925</v>
+      </c>
+      <c r="E8" t="s">
+        <v>463</v>
       </c>
     </row>
   </sheetData>

</xml_diff>